<commit_message>
Agregar gastos iO del 27 y 28 de septiembre
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Un1EUwZaDgQpX57Ncqbdo
</commit_message>
<xml_diff>
--- a/Seguimiento_Gastos.xlsx
+++ b/Seguimiento_Gastos.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gastos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gastos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Léeme" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -791,11 +791,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
+      <c r="A9" s="5" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>APPARKA APS</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>iO</t>
+        </is>
+      </c>
       <c r="F9" s="5">
         <f>IF(A9="","",IF(DAY(A9)&lt;=IF(E9="iO",25,10),DATE(YEAR(A9),MONTH(A9),IF(E9="iO",25,10)),DATE(YEAR(A9),MONTH(A9)+1,IF(E9="iO",25,10))))</f>
         <v/>
@@ -804,14 +820,34 @@
         <f>IF(F9="","",DATE(YEAR(F9),MONTH(F9)+1,IF(E9="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H9" s="6" t="n"/>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
+      <c r="A10" s="5" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>BESO FRANCES</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>iO</t>
+        </is>
+      </c>
       <c r="F10" s="5">
         <f>IF(A10="","",IF(DAY(A10)&lt;=IF(E10="iO",25,10),DATE(YEAR(A10),MONTH(A10),IF(E10="iO",25,10)),DATE(YEAR(A10),MONTH(A10)+1,IF(E10="iO",25,10))))</f>
         <v/>
@@ -820,14 +856,34 @@
         <f>IF(F10="","",DATE(YEAR(F10),MONTH(F10)+1,IF(E10="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H10" s="6" t="n"/>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
+      <c r="A11" s="5" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>PEAJES CASET</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>iO</t>
+        </is>
+      </c>
       <c r="F11" s="5">
         <f>IF(A11="","",IF(DAY(A11)&lt;=IF(E11="iO",25,10),DATE(YEAR(A11),MONTH(A11),IF(E11="iO",25,10)),DATE(YEAR(A11),MONTH(A11)+1,IF(E11="iO",25,10))))</f>
         <v/>
@@ -836,14 +892,34 @@
         <f>IF(F11="","",DATE(YEAR(F11),MONTH(F11)+1,IF(E11="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H11" s="6" t="n"/>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
+      <c r="A12" s="5" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>CEVICHERIA G</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>110</v>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>iO</t>
+        </is>
+      </c>
       <c r="F12" s="5">
         <f>IF(A12="","",IF(DAY(A12)&lt;=IF(E12="iO",25,10),DATE(YEAR(A12),MONTH(A12),IF(E12="iO",25,10)),DATE(YEAR(A12),MONTH(A12)+1,IF(E12="iO",25,10))))</f>
         <v/>
@@ -852,14 +928,34 @@
         <f>IF(F12="","",DATE(YEAR(F12),MONTH(F12)+1,IF(E12="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H12" s="6" t="n"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
+      <c r="A13" s="5" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>MERF PRIMAVE</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>iO</t>
+        </is>
+      </c>
       <c r="F13" s="5">
         <f>IF(A13="","",IF(DAY(A13)&lt;=IF(E13="iO",25,10),DATE(YEAR(A13),MONTH(A13),IF(E13="iO",25,10)),DATE(YEAR(A13),MONTH(A13)+1,IF(E13="iO",25,10))))</f>
         <v/>
@@ -868,14 +964,34 @@
         <f>IF(F13="","",DATE(YEAR(F13),MONTH(F13)+1,IF(E13="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H13" s="6" t="n"/>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
+      <c r="A14" s="5" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>CINEMARK</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>87</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>iO</t>
+        </is>
+      </c>
       <c r="F14" s="5">
         <f>IF(A14="","",IF(DAY(A14)&lt;=IF(E14="iO",25,10),DATE(YEAR(A14),MONTH(A14),IF(E14="iO",25,10)),DATE(YEAR(A14),MONTH(A14)+1,IF(E14="iO",25,10))))</f>
         <v/>
@@ -884,14 +1000,34 @@
         <f>IF(F14="","",DATE(YEAR(F14),MONTH(F14)+1,IF(E14="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H14" s="6" t="n"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
+      <c r="A15" s="5" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>190</v>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>iO</t>
+        </is>
+      </c>
       <c r="F15" s="5">
         <f>IF(A15="","",IF(DAY(A15)&lt;=IF(E15="iO",25,10),DATE(YEAR(A15),MONTH(A15),IF(E15="iO",25,10)),DATE(YEAR(A15),MONTH(A15)+1,IF(E15="iO",25,10))))</f>
         <v/>
@@ -900,7 +1036,11 @@
         <f>IF(F15="","",DATE(YEAR(F15),MONTH(F15)+1,IF(E15="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H15" s="6" t="n"/>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>

</xml_diff>

<commit_message>
Agregar gasto de pareja (148 USD, pago 20/11/2026)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Un1EUwZaDgQpX57Ncqbdo
</commit_message>
<xml_diff>
--- a/Seguimiento_Gastos.xlsx
+++ b/Seguimiento_Gastos.xlsx
@@ -1043,20 +1043,39 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
+      <c r="A16" s="5" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Gasto pareja</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>148</v>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Dólares</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>pareja</t>
+        </is>
+      </c>
       <c r="F16" s="5">
         <f>IF(A16="","",IF(DAY(A16)&lt;=IF(E16="iO",25,10),DATE(YEAR(A16),MONTH(A16),IF(E16="iO",25,10)),DATE(YEAR(A16),MONTH(A16)+1,IF(E16="iO",25,10))))</f>
         <v/>
       </c>
-      <c r="G16" s="5">
-        <f>IF(F16="","",DATE(YEAR(F16),MONTH(F16)+1,IF(E16="iO",12,5)))</f>
-        <v/>
-      </c>
-      <c r="H16" s="6" t="n"/>
+      <c r="G16" s="5" t="n">
+        <v>46346</v>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -4005,7 +4024,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"iO,BBVA"</formula1>
+      <formula1>"iO,BBVA,pareja"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Soles,Dólares"</formula1>
@@ -4024,7 +4043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4090,6 +4109,21 @@
       </c>
       <c r="C6" s="12">
         <f>SUMIFS(Gastos!C:C,Gastos!G:G,A6,Gastos!E:E,B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11">
+        <f>DATE(2026,11,20)</f>
+        <v/>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>pareja</t>
+        </is>
+      </c>
+      <c r="C7" s="12">
+        <f>SUMIFS(Gastos!C:C,Gastos!G:G,A7,Gastos!E:E,B7)</f>
         <v/>
       </c>
     </row>
@@ -4104,7 +4138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -4241,6 +4275,13 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Tarjeta 'pareja': la fecha de pago se escribe a mano en la columna Fecha de Pago (no usa fórmula).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar segmentos de gasto y pestaña Segmentos con % de ingreso y aproximado al cierre
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Un1EUwZaDgQpX57Ncqbdo
</commit_message>
<xml_diff>
--- a/Seguimiento_Gastos.xlsx
+++ b/Seguimiento_Gastos.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Gastos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Léeme" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Segmentos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Léeme" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +58,25 @@
       <name val="Arial"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -87,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -104,6 +125,22 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -469,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:J200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -480,6 +517,8 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,6 +562,16 @@
           <t>Estado</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Segmento</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Monto S/</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -561,6 +610,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Suscripciones</t>
+        </is>
+      </c>
+      <c r="J2" s="7">
+        <f>IF(C2="","",IF(D2="Dólares",C2*Segmentos!$B$4,C2))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -599,6 +657,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="J3" s="7">
+        <f>IF(C3="","",IF(D3="Dólares",C3*Segmentos!$B$4,C3))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -637,6 +704,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="J4" s="7">
+        <f>IF(C4="","",IF(D4="Dólares",C4*Segmentos!$B$4,C4))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -675,6 +751,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="J5" s="7">
+        <f>IF(C5="","",IF(D5="Dólares",C5*Segmentos!$B$4,C5))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -713,6 +798,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="J6" s="7">
+        <f>IF(C6="","",IF(D6="Dólares",C6*Segmentos!$B$4,C6))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -751,6 +845,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="J7" s="7">
+        <f>IF(C7="","",IF(D7="Dólares",C7*Segmentos!$B$4,C7))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -788,6 +891,15 @@
         <is>
           <t>Pendiente</t>
         </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="J8" s="7">
+        <f>IF(C8="","",IF(D8="Dólares",C8*Segmentos!$B$4,C8))</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -825,6 +937,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="J9" s="7">
+        <f>IF(C9="","",IF(D9="Dólares",C9*Segmentos!$B$4,C9))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -861,6 +982,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="J10" s="7">
+        <f>IF(C10="","",IF(D10="Dólares",C10*Segmentos!$B$4,C10))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -897,6 +1027,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="J11" s="7">
+        <f>IF(C11="","",IF(D11="Dólares",C11*Segmentos!$B$4,C11))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -933,6 +1072,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="J12" s="7">
+        <f>IF(C12="","",IF(D12="Dólares",C12*Segmentos!$B$4,C12))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -969,6 +1117,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="J13" s="7">
+        <f>IF(C13="","",IF(D13="Dólares",C13*Segmentos!$B$4,C13))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1005,6 +1162,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Ocio</t>
+        </is>
+      </c>
+      <c r="J14" s="7">
+        <f>IF(C14="","",IF(D14="Dólares",C14*Segmentos!$B$4,C14))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -1041,6 +1207,15 @@
           <t>Pendiente</t>
         </is>
       </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Ropa y compras</t>
+        </is>
+      </c>
+      <c r="J15" s="7">
+        <f>IF(C15="","",IF(D15="Dólares",C15*Segmentos!$B$4,C15))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -1075,6 +1250,15 @@
         <is>
           <t>Pendiente</t>
         </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="J16" s="7">
+        <f>IF(C16="","",IF(D16="Dólares",C16*Segmentos!$B$4,C16))</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1092,6 +1276,11 @@
         <v/>
       </c>
       <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="7">
+        <f>IF(C17="","",IF(D17="Dólares",C17*Segmentos!$B$4,C17))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -1108,6 +1297,11 @@
         <v/>
       </c>
       <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="7">
+        <f>IF(C18="","",IF(D18="Dólares",C18*Segmentos!$B$4,C18))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -1124,6 +1318,11 @@
         <v/>
       </c>
       <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="7">
+        <f>IF(C19="","",IF(D19="Dólares",C19*Segmentos!$B$4,C19))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
@@ -1140,6 +1339,11 @@
         <v/>
       </c>
       <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="7">
+        <f>IF(C20="","",IF(D20="Dólares",C20*Segmentos!$B$4,C20))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
@@ -1156,6 +1360,11 @@
         <v/>
       </c>
       <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+      <c r="J21" s="7">
+        <f>IF(C21="","",IF(D21="Dólares",C21*Segmentos!$B$4,C21))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
@@ -1172,6 +1381,11 @@
         <v/>
       </c>
       <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="7">
+        <f>IF(C22="","",IF(D22="Dólares",C22*Segmentos!$B$4,C22))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1188,6 +1402,11 @@
         <v/>
       </c>
       <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="7">
+        <f>IF(C23="","",IF(D23="Dólares",C23*Segmentos!$B$4,C23))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
@@ -1204,6 +1423,11 @@
         <v/>
       </c>
       <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
+      <c r="J24" s="7">
+        <f>IF(C24="","",IF(D24="Dólares",C24*Segmentos!$B$4,C24))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -1220,6 +1444,11 @@
         <v/>
       </c>
       <c r="H25" s="6" t="n"/>
+      <c r="I25" s="6" t="n"/>
+      <c r="J25" s="7">
+        <f>IF(C25="","",IF(D25="Dólares",C25*Segmentos!$B$4,C25))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
@@ -1236,6 +1465,11 @@
         <v/>
       </c>
       <c r="H26" s="6" t="n"/>
+      <c r="I26" s="6" t="n"/>
+      <c r="J26" s="7">
+        <f>IF(C26="","",IF(D26="Dólares",C26*Segmentos!$B$4,C26))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
@@ -1252,6 +1486,11 @@
         <v/>
       </c>
       <c r="H27" s="6" t="n"/>
+      <c r="I27" s="6" t="n"/>
+      <c r="J27" s="7">
+        <f>IF(C27="","",IF(D27="Dólares",C27*Segmentos!$B$4,C27))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
@@ -1268,6 +1507,11 @@
         <v/>
       </c>
       <c r="H28" s="6" t="n"/>
+      <c r="I28" s="6" t="n"/>
+      <c r="J28" s="7">
+        <f>IF(C28="","",IF(D28="Dólares",C28*Segmentos!$B$4,C28))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -1284,6 +1528,11 @@
         <v/>
       </c>
       <c r="H29" s="6" t="n"/>
+      <c r="I29" s="6" t="n"/>
+      <c r="J29" s="7">
+        <f>IF(C29="","",IF(D29="Dólares",C29*Segmentos!$B$4,C29))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
@@ -1300,6 +1549,11 @@
         <v/>
       </c>
       <c r="H30" s="6" t="n"/>
+      <c r="I30" s="6" t="n"/>
+      <c r="J30" s="7">
+        <f>IF(C30="","",IF(D30="Dólares",C30*Segmentos!$B$4,C30))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -1316,6 +1570,11 @@
         <v/>
       </c>
       <c r="H31" s="6" t="n"/>
+      <c r="I31" s="6" t="n"/>
+      <c r="J31" s="7">
+        <f>IF(C31="","",IF(D31="Dólares",C31*Segmentos!$B$4,C31))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
@@ -1332,6 +1591,11 @@
         <v/>
       </c>
       <c r="H32" s="6" t="n"/>
+      <c r="I32" s="6" t="n"/>
+      <c r="J32" s="7">
+        <f>IF(C32="","",IF(D32="Dólares",C32*Segmentos!$B$4,C32))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -1348,6 +1612,11 @@
         <v/>
       </c>
       <c r="H33" s="6" t="n"/>
+      <c r="I33" s="6" t="n"/>
+      <c r="J33" s="7">
+        <f>IF(C33="","",IF(D33="Dólares",C33*Segmentos!$B$4,C33))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>
@@ -1364,6 +1633,11 @@
         <v/>
       </c>
       <c r="H34" s="6" t="n"/>
+      <c r="I34" s="6" t="n"/>
+      <c r="J34" s="7">
+        <f>IF(C34="","",IF(D34="Dólares",C34*Segmentos!$B$4,C34))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -1380,6 +1654,11 @@
         <v/>
       </c>
       <c r="H35" s="6" t="n"/>
+      <c r="I35" s="6" t="n"/>
+      <c r="J35" s="7">
+        <f>IF(C35="","",IF(D35="Dólares",C35*Segmentos!$B$4,C35))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n"/>
@@ -1396,6 +1675,11 @@
         <v/>
       </c>
       <c r="H36" s="6" t="n"/>
+      <c r="I36" s="6" t="n"/>
+      <c r="J36" s="7">
+        <f>IF(C36="","",IF(D36="Dólares",C36*Segmentos!$B$4,C36))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -1412,6 +1696,11 @@
         <v/>
       </c>
       <c r="H37" s="6" t="n"/>
+      <c r="I37" s="6" t="n"/>
+      <c r="J37" s="7">
+        <f>IF(C37="","",IF(D37="Dólares",C37*Segmentos!$B$4,C37))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
@@ -1428,6 +1717,11 @@
         <v/>
       </c>
       <c r="H38" s="6" t="n"/>
+      <c r="I38" s="6" t="n"/>
+      <c r="J38" s="7">
+        <f>IF(C38="","",IF(D38="Dólares",C38*Segmentos!$B$4,C38))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -1444,6 +1738,11 @@
         <v/>
       </c>
       <c r="H39" s="6" t="n"/>
+      <c r="I39" s="6" t="n"/>
+      <c r="J39" s="7">
+        <f>IF(C39="","",IF(D39="Dólares",C39*Segmentos!$B$4,C39))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n"/>
@@ -1460,6 +1759,11 @@
         <v/>
       </c>
       <c r="H40" s="6" t="n"/>
+      <c r="I40" s="6" t="n"/>
+      <c r="J40" s="7">
+        <f>IF(C40="","",IF(D40="Dólares",C40*Segmentos!$B$4,C40))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -1476,6 +1780,11 @@
         <v/>
       </c>
       <c r="H41" s="6" t="n"/>
+      <c r="I41" s="6" t="n"/>
+      <c r="J41" s="7">
+        <f>IF(C41="","",IF(D41="Dólares",C41*Segmentos!$B$4,C41))</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
@@ -1492,6 +1801,11 @@
         <v/>
       </c>
       <c r="H42" s="6" t="n"/>
+      <c r="I42" s="6" t="n"/>
+      <c r="J42" s="7">
+        <f>IF(C42="","",IF(D42="Dólares",C42*Segmentos!$B$4,C42))</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -1508,6 +1822,11 @@
         <v/>
       </c>
       <c r="H43" s="6" t="n"/>
+      <c r="I43" s="6" t="n"/>
+      <c r="J43" s="7">
+        <f>IF(C43="","",IF(D43="Dólares",C43*Segmentos!$B$4,C43))</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
@@ -1524,6 +1843,11 @@
         <v/>
       </c>
       <c r="H44" s="6" t="n"/>
+      <c r="I44" s="6" t="n"/>
+      <c r="J44" s="7">
+        <f>IF(C44="","",IF(D44="Dólares",C44*Segmentos!$B$4,C44))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -1540,6 +1864,11 @@
         <v/>
       </c>
       <c r="H45" s="6" t="n"/>
+      <c r="I45" s="6" t="n"/>
+      <c r="J45" s="7">
+        <f>IF(C45="","",IF(D45="Dólares",C45*Segmentos!$B$4,C45))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n"/>
@@ -1556,6 +1885,11 @@
         <v/>
       </c>
       <c r="H46" s="6" t="n"/>
+      <c r="I46" s="6" t="n"/>
+      <c r="J46" s="7">
+        <f>IF(C46="","",IF(D46="Dólares",C46*Segmentos!$B$4,C46))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -1572,6 +1906,11 @@
         <v/>
       </c>
       <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="n"/>
+      <c r="J47" s="7">
+        <f>IF(C47="","",IF(D47="Dólares",C47*Segmentos!$B$4,C47))</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
@@ -1588,6 +1927,11 @@
         <v/>
       </c>
       <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="n"/>
+      <c r="J48" s="7">
+        <f>IF(C48="","",IF(D48="Dólares",C48*Segmentos!$B$4,C48))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -1604,6 +1948,11 @@
         <v/>
       </c>
       <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="n"/>
+      <c r="J49" s="7">
+        <f>IF(C49="","",IF(D49="Dólares",C49*Segmentos!$B$4,C49))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n"/>
@@ -1620,6 +1969,11 @@
         <v/>
       </c>
       <c r="H50" s="6" t="n"/>
+      <c r="I50" s="6" t="n"/>
+      <c r="J50" s="7">
+        <f>IF(C50="","",IF(D50="Dólares",C50*Segmentos!$B$4,C50))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -1636,6 +1990,11 @@
         <v/>
       </c>
       <c r="H51" s="6" t="n"/>
+      <c r="I51" s="6" t="n"/>
+      <c r="J51" s="7">
+        <f>IF(C51="","",IF(D51="Dólares",C51*Segmentos!$B$4,C51))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
@@ -1652,6 +2011,11 @@
         <v/>
       </c>
       <c r="H52" s="6" t="n"/>
+      <c r="I52" s="6" t="n"/>
+      <c r="J52" s="7">
+        <f>IF(C52="","",IF(D52="Dólares",C52*Segmentos!$B$4,C52))</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -1668,6 +2032,11 @@
         <v/>
       </c>
       <c r="H53" s="6" t="n"/>
+      <c r="I53" s="6" t="n"/>
+      <c r="J53" s="7">
+        <f>IF(C53="","",IF(D53="Dólares",C53*Segmentos!$B$4,C53))</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
@@ -1684,6 +2053,11 @@
         <v/>
       </c>
       <c r="H54" s="6" t="n"/>
+      <c r="I54" s="6" t="n"/>
+      <c r="J54" s="7">
+        <f>IF(C54="","",IF(D54="Dólares",C54*Segmentos!$B$4,C54))</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
@@ -1700,6 +2074,11 @@
         <v/>
       </c>
       <c r="H55" s="6" t="n"/>
+      <c r="I55" s="6" t="n"/>
+      <c r="J55" s="7">
+        <f>IF(C55="","",IF(D55="Dólares",C55*Segmentos!$B$4,C55))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n"/>
@@ -1716,6 +2095,11 @@
         <v/>
       </c>
       <c r="H56" s="6" t="n"/>
+      <c r="I56" s="6" t="n"/>
+      <c r="J56" s="7">
+        <f>IF(C56="","",IF(D56="Dólares",C56*Segmentos!$B$4,C56))</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
@@ -1732,6 +2116,11 @@
         <v/>
       </c>
       <c r="H57" s="6" t="n"/>
+      <c r="I57" s="6" t="n"/>
+      <c r="J57" s="7">
+        <f>IF(C57="","",IF(D57="Dólares",C57*Segmentos!$B$4,C57))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n"/>
@@ -1748,6 +2137,11 @@
         <v/>
       </c>
       <c r="H58" s="6" t="n"/>
+      <c r="I58" s="6" t="n"/>
+      <c r="J58" s="7">
+        <f>IF(C58="","",IF(D58="Dólares",C58*Segmentos!$B$4,C58))</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
@@ -1764,6 +2158,11 @@
         <v/>
       </c>
       <c r="H59" s="6" t="n"/>
+      <c r="I59" s="6" t="n"/>
+      <c r="J59" s="7">
+        <f>IF(C59="","",IF(D59="Dólares",C59*Segmentos!$B$4,C59))</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
@@ -1780,6 +2179,11 @@
         <v/>
       </c>
       <c r="H60" s="6" t="n"/>
+      <c r="I60" s="6" t="n"/>
+      <c r="J60" s="7">
+        <f>IF(C60="","",IF(D60="Dólares",C60*Segmentos!$B$4,C60))</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n"/>
@@ -1796,6 +2200,11 @@
         <v/>
       </c>
       <c r="H61" s="6" t="n"/>
+      <c r="I61" s="6" t="n"/>
+      <c r="J61" s="7">
+        <f>IF(C61="","",IF(D61="Dólares",C61*Segmentos!$B$4,C61))</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n"/>
@@ -1812,6 +2221,11 @@
         <v/>
       </c>
       <c r="H62" s="6" t="n"/>
+      <c r="I62" s="6" t="n"/>
+      <c r="J62" s="7">
+        <f>IF(C62="","",IF(D62="Dólares",C62*Segmentos!$B$4,C62))</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n"/>
@@ -1828,6 +2242,11 @@
         <v/>
       </c>
       <c r="H63" s="6" t="n"/>
+      <c r="I63" s="6" t="n"/>
+      <c r="J63" s="7">
+        <f>IF(C63="","",IF(D63="Dólares",C63*Segmentos!$B$4,C63))</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n"/>
@@ -1844,6 +2263,11 @@
         <v/>
       </c>
       <c r="H64" s="6" t="n"/>
+      <c r="I64" s="6" t="n"/>
+      <c r="J64" s="7">
+        <f>IF(C64="","",IF(D64="Dólares",C64*Segmentos!$B$4,C64))</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n"/>
@@ -1860,6 +2284,11 @@
         <v/>
       </c>
       <c r="H65" s="6" t="n"/>
+      <c r="I65" s="6" t="n"/>
+      <c r="J65" s="7">
+        <f>IF(C65="","",IF(D65="Dólares",C65*Segmentos!$B$4,C65))</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n"/>
@@ -1876,6 +2305,11 @@
         <v/>
       </c>
       <c r="H66" s="6" t="n"/>
+      <c r="I66" s="6" t="n"/>
+      <c r="J66" s="7">
+        <f>IF(C66="","",IF(D66="Dólares",C66*Segmentos!$B$4,C66))</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n"/>
@@ -1892,6 +2326,11 @@
         <v/>
       </c>
       <c r="H67" s="6" t="n"/>
+      <c r="I67" s="6" t="n"/>
+      <c r="J67" s="7">
+        <f>IF(C67="","",IF(D67="Dólares",C67*Segmentos!$B$4,C67))</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n"/>
@@ -1908,6 +2347,11 @@
         <v/>
       </c>
       <c r="H68" s="6" t="n"/>
+      <c r="I68" s="6" t="n"/>
+      <c r="J68" s="7">
+        <f>IF(C68="","",IF(D68="Dólares",C68*Segmentos!$B$4,C68))</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n"/>
@@ -1924,6 +2368,11 @@
         <v/>
       </c>
       <c r="H69" s="6" t="n"/>
+      <c r="I69" s="6" t="n"/>
+      <c r="J69" s="7">
+        <f>IF(C69="","",IF(D69="Dólares",C69*Segmentos!$B$4,C69))</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n"/>
@@ -1940,6 +2389,11 @@
         <v/>
       </c>
       <c r="H70" s="6" t="n"/>
+      <c r="I70" s="6" t="n"/>
+      <c r="J70" s="7">
+        <f>IF(C70="","",IF(D70="Dólares",C70*Segmentos!$B$4,C70))</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n"/>
@@ -1956,6 +2410,11 @@
         <v/>
       </c>
       <c r="H71" s="6" t="n"/>
+      <c r="I71" s="6" t="n"/>
+      <c r="J71" s="7">
+        <f>IF(C71="","",IF(D71="Dólares",C71*Segmentos!$B$4,C71))</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n"/>
@@ -1972,6 +2431,11 @@
         <v/>
       </c>
       <c r="H72" s="6" t="n"/>
+      <c r="I72" s="6" t="n"/>
+      <c r="J72" s="7">
+        <f>IF(C72="","",IF(D72="Dólares",C72*Segmentos!$B$4,C72))</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n"/>
@@ -1988,6 +2452,11 @@
         <v/>
       </c>
       <c r="H73" s="6" t="n"/>
+      <c r="I73" s="6" t="n"/>
+      <c r="J73" s="7">
+        <f>IF(C73="","",IF(D73="Dólares",C73*Segmentos!$B$4,C73))</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n"/>
@@ -2004,6 +2473,11 @@
         <v/>
       </c>
       <c r="H74" s="6" t="n"/>
+      <c r="I74" s="6" t="n"/>
+      <c r="J74" s="7">
+        <f>IF(C74="","",IF(D74="Dólares",C74*Segmentos!$B$4,C74))</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n"/>
@@ -2020,6 +2494,11 @@
         <v/>
       </c>
       <c r="H75" s="6" t="n"/>
+      <c r="I75" s="6" t="n"/>
+      <c r="J75" s="7">
+        <f>IF(C75="","",IF(D75="Dólares",C75*Segmentos!$B$4,C75))</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n"/>
@@ -2036,6 +2515,11 @@
         <v/>
       </c>
       <c r="H76" s="6" t="n"/>
+      <c r="I76" s="6" t="n"/>
+      <c r="J76" s="7">
+        <f>IF(C76="","",IF(D76="Dólares",C76*Segmentos!$B$4,C76))</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n"/>
@@ -2052,6 +2536,11 @@
         <v/>
       </c>
       <c r="H77" s="6" t="n"/>
+      <c r="I77" s="6" t="n"/>
+      <c r="J77" s="7">
+        <f>IF(C77="","",IF(D77="Dólares",C77*Segmentos!$B$4,C77))</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n"/>
@@ -2068,6 +2557,11 @@
         <v/>
       </c>
       <c r="H78" s="6" t="n"/>
+      <c r="I78" s="6" t="n"/>
+      <c r="J78" s="7">
+        <f>IF(C78="","",IF(D78="Dólares",C78*Segmentos!$B$4,C78))</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n"/>
@@ -2084,6 +2578,11 @@
         <v/>
       </c>
       <c r="H79" s="6" t="n"/>
+      <c r="I79" s="6" t="n"/>
+      <c r="J79" s="7">
+        <f>IF(C79="","",IF(D79="Dólares",C79*Segmentos!$B$4,C79))</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n"/>
@@ -2100,6 +2599,11 @@
         <v/>
       </c>
       <c r="H80" s="6" t="n"/>
+      <c r="I80" s="6" t="n"/>
+      <c r="J80" s="7">
+        <f>IF(C80="","",IF(D80="Dólares",C80*Segmentos!$B$4,C80))</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n"/>
@@ -2116,6 +2620,11 @@
         <v/>
       </c>
       <c r="H81" s="6" t="n"/>
+      <c r="I81" s="6" t="n"/>
+      <c r="J81" s="7">
+        <f>IF(C81="","",IF(D81="Dólares",C81*Segmentos!$B$4,C81))</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n"/>
@@ -2132,6 +2641,11 @@
         <v/>
       </c>
       <c r="H82" s="6" t="n"/>
+      <c r="I82" s="6" t="n"/>
+      <c r="J82" s="7">
+        <f>IF(C82="","",IF(D82="Dólares",C82*Segmentos!$B$4,C82))</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n"/>
@@ -2148,6 +2662,11 @@
         <v/>
       </c>
       <c r="H83" s="6" t="n"/>
+      <c r="I83" s="6" t="n"/>
+      <c r="J83" s="7">
+        <f>IF(C83="","",IF(D83="Dólares",C83*Segmentos!$B$4,C83))</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n"/>
@@ -2164,6 +2683,11 @@
         <v/>
       </c>
       <c r="H84" s="6" t="n"/>
+      <c r="I84" s="6" t="n"/>
+      <c r="J84" s="7">
+        <f>IF(C84="","",IF(D84="Dólares",C84*Segmentos!$B$4,C84))</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n"/>
@@ -2180,6 +2704,11 @@
         <v/>
       </c>
       <c r="H85" s="6" t="n"/>
+      <c r="I85" s="6" t="n"/>
+      <c r="J85" s="7">
+        <f>IF(C85="","",IF(D85="Dólares",C85*Segmentos!$B$4,C85))</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n"/>
@@ -2196,6 +2725,11 @@
         <v/>
       </c>
       <c r="H86" s="6" t="n"/>
+      <c r="I86" s="6" t="n"/>
+      <c r="J86" s="7">
+        <f>IF(C86="","",IF(D86="Dólares",C86*Segmentos!$B$4,C86))</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n"/>
@@ -2212,6 +2746,11 @@
         <v/>
       </c>
       <c r="H87" s="6" t="n"/>
+      <c r="I87" s="6" t="n"/>
+      <c r="J87" s="7">
+        <f>IF(C87="","",IF(D87="Dólares",C87*Segmentos!$B$4,C87))</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n"/>
@@ -2228,6 +2767,11 @@
         <v/>
       </c>
       <c r="H88" s="6" t="n"/>
+      <c r="I88" s="6" t="n"/>
+      <c r="J88" s="7">
+        <f>IF(C88="","",IF(D88="Dólares",C88*Segmentos!$B$4,C88))</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n"/>
@@ -2244,6 +2788,11 @@
         <v/>
       </c>
       <c r="H89" s="6" t="n"/>
+      <c r="I89" s="6" t="n"/>
+      <c r="J89" s="7">
+        <f>IF(C89="","",IF(D89="Dólares",C89*Segmentos!$B$4,C89))</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n"/>
@@ -2260,6 +2809,11 @@
         <v/>
       </c>
       <c r="H90" s="6" t="n"/>
+      <c r="I90" s="6" t="n"/>
+      <c r="J90" s="7">
+        <f>IF(C90="","",IF(D90="Dólares",C90*Segmentos!$B$4,C90))</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n"/>
@@ -2276,6 +2830,11 @@
         <v/>
       </c>
       <c r="H91" s="6" t="n"/>
+      <c r="I91" s="6" t="n"/>
+      <c r="J91" s="7">
+        <f>IF(C91="","",IF(D91="Dólares",C91*Segmentos!$B$4,C91))</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="n"/>
@@ -2292,6 +2851,11 @@
         <v/>
       </c>
       <c r="H92" s="6" t="n"/>
+      <c r="I92" s="6" t="n"/>
+      <c r="J92" s="7">
+        <f>IF(C92="","",IF(D92="Dólares",C92*Segmentos!$B$4,C92))</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="n"/>
@@ -2308,6 +2872,11 @@
         <v/>
       </c>
       <c r="H93" s="6" t="n"/>
+      <c r="I93" s="6" t="n"/>
+      <c r="J93" s="7">
+        <f>IF(C93="","",IF(D93="Dólares",C93*Segmentos!$B$4,C93))</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n"/>
@@ -2324,6 +2893,11 @@
         <v/>
       </c>
       <c r="H94" s="6" t="n"/>
+      <c r="I94" s="6" t="n"/>
+      <c r="J94" s="7">
+        <f>IF(C94="","",IF(D94="Dólares",C94*Segmentos!$B$4,C94))</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="n"/>
@@ -2340,6 +2914,11 @@
         <v/>
       </c>
       <c r="H95" s="6" t="n"/>
+      <c r="I95" s="6" t="n"/>
+      <c r="J95" s="7">
+        <f>IF(C95="","",IF(D95="Dólares",C95*Segmentos!$B$4,C95))</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n"/>
@@ -2356,6 +2935,11 @@
         <v/>
       </c>
       <c r="H96" s="6" t="n"/>
+      <c r="I96" s="6" t="n"/>
+      <c r="J96" s="7">
+        <f>IF(C96="","",IF(D96="Dólares",C96*Segmentos!$B$4,C96))</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n"/>
@@ -2372,6 +2956,11 @@
         <v/>
       </c>
       <c r="H97" s="6" t="n"/>
+      <c r="I97" s="6" t="n"/>
+      <c r="J97" s="7">
+        <f>IF(C97="","",IF(D97="Dólares",C97*Segmentos!$B$4,C97))</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n"/>
@@ -2388,6 +2977,11 @@
         <v/>
       </c>
       <c r="H98" s="6" t="n"/>
+      <c r="I98" s="6" t="n"/>
+      <c r="J98" s="7">
+        <f>IF(C98="","",IF(D98="Dólares",C98*Segmentos!$B$4,C98))</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="n"/>
@@ -2404,6 +2998,11 @@
         <v/>
       </c>
       <c r="H99" s="6" t="n"/>
+      <c r="I99" s="6" t="n"/>
+      <c r="J99" s="7">
+        <f>IF(C99="","",IF(D99="Dólares",C99*Segmentos!$B$4,C99))</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="n"/>
@@ -2420,6 +3019,11 @@
         <v/>
       </c>
       <c r="H100" s="6" t="n"/>
+      <c r="I100" s="6" t="n"/>
+      <c r="J100" s="7">
+        <f>IF(C100="","",IF(D100="Dólares",C100*Segmentos!$B$4,C100))</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="n"/>
@@ -2436,6 +3040,11 @@
         <v/>
       </c>
       <c r="H101" s="6" t="n"/>
+      <c r="I101" s="6" t="n"/>
+      <c r="J101" s="7">
+        <f>IF(C101="","",IF(D101="Dólares",C101*Segmentos!$B$4,C101))</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n"/>
@@ -2452,6 +3061,11 @@
         <v/>
       </c>
       <c r="H102" s="6" t="n"/>
+      <c r="I102" s="6" t="n"/>
+      <c r="J102" s="7">
+        <f>IF(C102="","",IF(D102="Dólares",C102*Segmentos!$B$4,C102))</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="n"/>
@@ -2468,6 +3082,11 @@
         <v/>
       </c>
       <c r="H103" s="6" t="n"/>
+      <c r="I103" s="6" t="n"/>
+      <c r="J103" s="7">
+        <f>IF(C103="","",IF(D103="Dólares",C103*Segmentos!$B$4,C103))</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n"/>
@@ -2484,6 +3103,11 @@
         <v/>
       </c>
       <c r="H104" s="6" t="n"/>
+      <c r="I104" s="6" t="n"/>
+      <c r="J104" s="7">
+        <f>IF(C104="","",IF(D104="Dólares",C104*Segmentos!$B$4,C104))</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="n"/>
@@ -2500,6 +3124,11 @@
         <v/>
       </c>
       <c r="H105" s="6" t="n"/>
+      <c r="I105" s="6" t="n"/>
+      <c r="J105" s="7">
+        <f>IF(C105="","",IF(D105="Dólares",C105*Segmentos!$B$4,C105))</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n"/>
@@ -2516,6 +3145,11 @@
         <v/>
       </c>
       <c r="H106" s="6" t="n"/>
+      <c r="I106" s="6" t="n"/>
+      <c r="J106" s="7">
+        <f>IF(C106="","",IF(D106="Dólares",C106*Segmentos!$B$4,C106))</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n"/>
@@ -2532,6 +3166,11 @@
         <v/>
       </c>
       <c r="H107" s="6" t="n"/>
+      <c r="I107" s="6" t="n"/>
+      <c r="J107" s="7">
+        <f>IF(C107="","",IF(D107="Dólares",C107*Segmentos!$B$4,C107))</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n"/>
@@ -2548,6 +3187,11 @@
         <v/>
       </c>
       <c r="H108" s="6" t="n"/>
+      <c r="I108" s="6" t="n"/>
+      <c r="J108" s="7">
+        <f>IF(C108="","",IF(D108="Dólares",C108*Segmentos!$B$4,C108))</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="n"/>
@@ -2564,6 +3208,11 @@
         <v/>
       </c>
       <c r="H109" s="6" t="n"/>
+      <c r="I109" s="6" t="n"/>
+      <c r="J109" s="7">
+        <f>IF(C109="","",IF(D109="Dólares",C109*Segmentos!$B$4,C109))</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n"/>
@@ -2580,6 +3229,11 @@
         <v/>
       </c>
       <c r="H110" s="6" t="n"/>
+      <c r="I110" s="6" t="n"/>
+      <c r="J110" s="7">
+        <f>IF(C110="","",IF(D110="Dólares",C110*Segmentos!$B$4,C110))</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n"/>
@@ -2596,6 +3250,11 @@
         <v/>
       </c>
       <c r="H111" s="6" t="n"/>
+      <c r="I111" s="6" t="n"/>
+      <c r="J111" s="7">
+        <f>IF(C111="","",IF(D111="Dólares",C111*Segmentos!$B$4,C111))</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="n"/>
@@ -2612,6 +3271,11 @@
         <v/>
       </c>
       <c r="H112" s="6" t="n"/>
+      <c r="I112" s="6" t="n"/>
+      <c r="J112" s="7">
+        <f>IF(C112="","",IF(D112="Dólares",C112*Segmentos!$B$4,C112))</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="n"/>
@@ -2628,6 +3292,11 @@
         <v/>
       </c>
       <c r="H113" s="6" t="n"/>
+      <c r="I113" s="6" t="n"/>
+      <c r="J113" s="7">
+        <f>IF(C113="","",IF(D113="Dólares",C113*Segmentos!$B$4,C113))</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="n"/>
@@ -2644,6 +3313,11 @@
         <v/>
       </c>
       <c r="H114" s="6" t="n"/>
+      <c r="I114" s="6" t="n"/>
+      <c r="J114" s="7">
+        <f>IF(C114="","",IF(D114="Dólares",C114*Segmentos!$B$4,C114))</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="n"/>
@@ -2660,6 +3334,11 @@
         <v/>
       </c>
       <c r="H115" s="6" t="n"/>
+      <c r="I115" s="6" t="n"/>
+      <c r="J115" s="7">
+        <f>IF(C115="","",IF(D115="Dólares",C115*Segmentos!$B$4,C115))</f>
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n"/>
@@ -2676,6 +3355,11 @@
         <v/>
       </c>
       <c r="H116" s="6" t="n"/>
+      <c r="I116" s="6" t="n"/>
+      <c r="J116" s="7">
+        <f>IF(C116="","",IF(D116="Dólares",C116*Segmentos!$B$4,C116))</f>
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="n"/>
@@ -2692,6 +3376,11 @@
         <v/>
       </c>
       <c r="H117" s="6" t="n"/>
+      <c r="I117" s="6" t="n"/>
+      <c r="J117" s="7">
+        <f>IF(C117="","",IF(D117="Dólares",C117*Segmentos!$B$4,C117))</f>
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="n"/>
@@ -2708,6 +3397,11 @@
         <v/>
       </c>
       <c r="H118" s="6" t="n"/>
+      <c r="I118" s="6" t="n"/>
+      <c r="J118" s="7">
+        <f>IF(C118="","",IF(D118="Dólares",C118*Segmentos!$B$4,C118))</f>
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n"/>
@@ -2724,6 +3418,11 @@
         <v/>
       </c>
       <c r="H119" s="6" t="n"/>
+      <c r="I119" s="6" t="n"/>
+      <c r="J119" s="7">
+        <f>IF(C119="","",IF(D119="Dólares",C119*Segmentos!$B$4,C119))</f>
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n"/>
@@ -2740,6 +3439,11 @@
         <v/>
       </c>
       <c r="H120" s="6" t="n"/>
+      <c r="I120" s="6" t="n"/>
+      <c r="J120" s="7">
+        <f>IF(C120="","",IF(D120="Dólares",C120*Segmentos!$B$4,C120))</f>
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n"/>
@@ -2756,6 +3460,11 @@
         <v/>
       </c>
       <c r="H121" s="6" t="n"/>
+      <c r="I121" s="6" t="n"/>
+      <c r="J121" s="7">
+        <f>IF(C121="","",IF(D121="Dólares",C121*Segmentos!$B$4,C121))</f>
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="n"/>
@@ -2772,6 +3481,11 @@
         <v/>
       </c>
       <c r="H122" s="6" t="n"/>
+      <c r="I122" s="6" t="n"/>
+      <c r="J122" s="7">
+        <f>IF(C122="","",IF(D122="Dólares",C122*Segmentos!$B$4,C122))</f>
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="n"/>
@@ -2788,6 +3502,11 @@
         <v/>
       </c>
       <c r="H123" s="6" t="n"/>
+      <c r="I123" s="6" t="n"/>
+      <c r="J123" s="7">
+        <f>IF(C123="","",IF(D123="Dólares",C123*Segmentos!$B$4,C123))</f>
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="n"/>
@@ -2804,6 +3523,11 @@
         <v/>
       </c>
       <c r="H124" s="6" t="n"/>
+      <c r="I124" s="6" t="n"/>
+      <c r="J124" s="7">
+        <f>IF(C124="","",IF(D124="Dólares",C124*Segmentos!$B$4,C124))</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="n"/>
@@ -2820,6 +3544,11 @@
         <v/>
       </c>
       <c r="H125" s="6" t="n"/>
+      <c r="I125" s="6" t="n"/>
+      <c r="J125" s="7">
+        <f>IF(C125="","",IF(D125="Dólares",C125*Segmentos!$B$4,C125))</f>
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="5" t="n"/>
@@ -2836,6 +3565,11 @@
         <v/>
       </c>
       <c r="H126" s="6" t="n"/>
+      <c r="I126" s="6" t="n"/>
+      <c r="J126" s="7">
+        <f>IF(C126="","",IF(D126="Dólares",C126*Segmentos!$B$4,C126))</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="n"/>
@@ -2852,6 +3586,11 @@
         <v/>
       </c>
       <c r="H127" s="6" t="n"/>
+      <c r="I127" s="6" t="n"/>
+      <c r="J127" s="7">
+        <f>IF(C127="","",IF(D127="Dólares",C127*Segmentos!$B$4,C127))</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="n"/>
@@ -2868,6 +3607,11 @@
         <v/>
       </c>
       <c r="H128" s="6" t="n"/>
+      <c r="I128" s="6" t="n"/>
+      <c r="J128" s="7">
+        <f>IF(C128="","",IF(D128="Dólares",C128*Segmentos!$B$4,C128))</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="n"/>
@@ -2884,6 +3628,11 @@
         <v/>
       </c>
       <c r="H129" s="6" t="n"/>
+      <c r="I129" s="6" t="n"/>
+      <c r="J129" s="7">
+        <f>IF(C129="","",IF(D129="Dólares",C129*Segmentos!$B$4,C129))</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n"/>
@@ -2900,6 +3649,11 @@
         <v/>
       </c>
       <c r="H130" s="6" t="n"/>
+      <c r="I130" s="6" t="n"/>
+      <c r="J130" s="7">
+        <f>IF(C130="","",IF(D130="Dólares",C130*Segmentos!$B$4,C130))</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="5" t="n"/>
@@ -2916,6 +3670,11 @@
         <v/>
       </c>
       <c r="H131" s="6" t="n"/>
+      <c r="I131" s="6" t="n"/>
+      <c r="J131" s="7">
+        <f>IF(C131="","",IF(D131="Dólares",C131*Segmentos!$B$4,C131))</f>
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="5" t="n"/>
@@ -2932,6 +3691,11 @@
         <v/>
       </c>
       <c r="H132" s="6" t="n"/>
+      <c r="I132" s="6" t="n"/>
+      <c r="J132" s="7">
+        <f>IF(C132="","",IF(D132="Dólares",C132*Segmentos!$B$4,C132))</f>
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="5" t="n"/>
@@ -2948,6 +3712,11 @@
         <v/>
       </c>
       <c r="H133" s="6" t="n"/>
+      <c r="I133" s="6" t="n"/>
+      <c r="J133" s="7">
+        <f>IF(C133="","",IF(D133="Dólares",C133*Segmentos!$B$4,C133))</f>
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="5" t="n"/>
@@ -2964,6 +3733,11 @@
         <v/>
       </c>
       <c r="H134" s="6" t="n"/>
+      <c r="I134" s="6" t="n"/>
+      <c r="J134" s="7">
+        <f>IF(C134="","",IF(D134="Dólares",C134*Segmentos!$B$4,C134))</f>
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="n"/>
@@ -2980,6 +3754,11 @@
         <v/>
       </c>
       <c r="H135" s="6" t="n"/>
+      <c r="I135" s="6" t="n"/>
+      <c r="J135" s="7">
+        <f>IF(C135="","",IF(D135="Dólares",C135*Segmentos!$B$4,C135))</f>
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n"/>
@@ -2996,6 +3775,11 @@
         <v/>
       </c>
       <c r="H136" s="6" t="n"/>
+      <c r="I136" s="6" t="n"/>
+      <c r="J136" s="7">
+        <f>IF(C136="","",IF(D136="Dólares",C136*Segmentos!$B$4,C136))</f>
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n"/>
@@ -3012,6 +3796,11 @@
         <v/>
       </c>
       <c r="H137" s="6" t="n"/>
+      <c r="I137" s="6" t="n"/>
+      <c r="J137" s="7">
+        <f>IF(C137="","",IF(D137="Dólares",C137*Segmentos!$B$4,C137))</f>
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="n"/>
@@ -3028,6 +3817,11 @@
         <v/>
       </c>
       <c r="H138" s="6" t="n"/>
+      <c r="I138" s="6" t="n"/>
+      <c r="J138" s="7">
+        <f>IF(C138="","",IF(D138="Dólares",C138*Segmentos!$B$4,C138))</f>
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="n"/>
@@ -3044,6 +3838,11 @@
         <v/>
       </c>
       <c r="H139" s="6" t="n"/>
+      <c r="I139" s="6" t="n"/>
+      <c r="J139" s="7">
+        <f>IF(C139="","",IF(D139="Dólares",C139*Segmentos!$B$4,C139))</f>
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="n"/>
@@ -3060,6 +3859,11 @@
         <v/>
       </c>
       <c r="H140" s="6" t="n"/>
+      <c r="I140" s="6" t="n"/>
+      <c r="J140" s="7">
+        <f>IF(C140="","",IF(D140="Dólares",C140*Segmentos!$B$4,C140))</f>
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="n"/>
@@ -3076,6 +3880,11 @@
         <v/>
       </c>
       <c r="H141" s="6" t="n"/>
+      <c r="I141" s="6" t="n"/>
+      <c r="J141" s="7">
+        <f>IF(C141="","",IF(D141="Dólares",C141*Segmentos!$B$4,C141))</f>
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="5" t="n"/>
@@ -3092,6 +3901,11 @@
         <v/>
       </c>
       <c r="H142" s="6" t="n"/>
+      <c r="I142" s="6" t="n"/>
+      <c r="J142" s="7">
+        <f>IF(C142="","",IF(D142="Dólares",C142*Segmentos!$B$4,C142))</f>
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="5" t="n"/>
@@ -3108,6 +3922,11 @@
         <v/>
       </c>
       <c r="H143" s="6" t="n"/>
+      <c r="I143" s="6" t="n"/>
+      <c r="J143" s="7">
+        <f>IF(C143="","",IF(D143="Dólares",C143*Segmentos!$B$4,C143))</f>
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n"/>
@@ -3124,6 +3943,11 @@
         <v/>
       </c>
       <c r="H144" s="6" t="n"/>
+      <c r="I144" s="6" t="n"/>
+      <c r="J144" s="7">
+        <f>IF(C144="","",IF(D144="Dólares",C144*Segmentos!$B$4,C144))</f>
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="n"/>
@@ -3140,6 +3964,11 @@
         <v/>
       </c>
       <c r="H145" s="6" t="n"/>
+      <c r="I145" s="6" t="n"/>
+      <c r="J145" s="7">
+        <f>IF(C145="","",IF(D145="Dólares",C145*Segmentos!$B$4,C145))</f>
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n"/>
@@ -3156,6 +3985,11 @@
         <v/>
       </c>
       <c r="H146" s="6" t="n"/>
+      <c r="I146" s="6" t="n"/>
+      <c r="J146" s="7">
+        <f>IF(C146="","",IF(D146="Dólares",C146*Segmentos!$B$4,C146))</f>
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n"/>
@@ -3172,6 +4006,11 @@
         <v/>
       </c>
       <c r="H147" s="6" t="n"/>
+      <c r="I147" s="6" t="n"/>
+      <c r="J147" s="7">
+        <f>IF(C147="","",IF(D147="Dólares",C147*Segmentos!$B$4,C147))</f>
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="5" t="n"/>
@@ -3188,6 +4027,11 @@
         <v/>
       </c>
       <c r="H148" s="6" t="n"/>
+      <c r="I148" s="6" t="n"/>
+      <c r="J148" s="7">
+        <f>IF(C148="","",IF(D148="Dólares",C148*Segmentos!$B$4,C148))</f>
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="n"/>
@@ -3204,6 +4048,11 @@
         <v/>
       </c>
       <c r="H149" s="6" t="n"/>
+      <c r="I149" s="6" t="n"/>
+      <c r="J149" s="7">
+        <f>IF(C149="","",IF(D149="Dólares",C149*Segmentos!$B$4,C149))</f>
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="5" t="n"/>
@@ -3220,6 +4069,11 @@
         <v/>
       </c>
       <c r="H150" s="6" t="n"/>
+      <c r="I150" s="6" t="n"/>
+      <c r="J150" s="7">
+        <f>IF(C150="","",IF(D150="Dólares",C150*Segmentos!$B$4,C150))</f>
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="5" t="n"/>
@@ -3236,6 +4090,11 @@
         <v/>
       </c>
       <c r="H151" s="6" t="n"/>
+      <c r="I151" s="6" t="n"/>
+      <c r="J151" s="7">
+        <f>IF(C151="","",IF(D151="Dólares",C151*Segmentos!$B$4,C151))</f>
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="5" t="n"/>
@@ -3252,6 +4111,11 @@
         <v/>
       </c>
       <c r="H152" s="6" t="n"/>
+      <c r="I152" s="6" t="n"/>
+      <c r="J152" s="7">
+        <f>IF(C152="","",IF(D152="Dólares",C152*Segmentos!$B$4,C152))</f>
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="n"/>
@@ -3268,6 +4132,11 @@
         <v/>
       </c>
       <c r="H153" s="6" t="n"/>
+      <c r="I153" s="6" t="n"/>
+      <c r="J153" s="7">
+        <f>IF(C153="","",IF(D153="Dólares",C153*Segmentos!$B$4,C153))</f>
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="5" t="n"/>
@@ -3284,6 +4153,11 @@
         <v/>
       </c>
       <c r="H154" s="6" t="n"/>
+      <c r="I154" s="6" t="n"/>
+      <c r="J154" s="7">
+        <f>IF(C154="","",IF(D154="Dólares",C154*Segmentos!$B$4,C154))</f>
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="n"/>
@@ -3300,6 +4174,11 @@
         <v/>
       </c>
       <c r="H155" s="6" t="n"/>
+      <c r="I155" s="6" t="n"/>
+      <c r="J155" s="7">
+        <f>IF(C155="","",IF(D155="Dólares",C155*Segmentos!$B$4,C155))</f>
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n"/>
@@ -3316,6 +4195,11 @@
         <v/>
       </c>
       <c r="H156" s="6" t="n"/>
+      <c r="I156" s="6" t="n"/>
+      <c r="J156" s="7">
+        <f>IF(C156="","",IF(D156="Dólares",C156*Segmentos!$B$4,C156))</f>
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="n"/>
@@ -3332,6 +4216,11 @@
         <v/>
       </c>
       <c r="H157" s="6" t="n"/>
+      <c r="I157" s="6" t="n"/>
+      <c r="J157" s="7">
+        <f>IF(C157="","",IF(D157="Dólares",C157*Segmentos!$B$4,C157))</f>
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="5" t="n"/>
@@ -3348,6 +4237,11 @@
         <v/>
       </c>
       <c r="H158" s="6" t="n"/>
+      <c r="I158" s="6" t="n"/>
+      <c r="J158" s="7">
+        <f>IF(C158="","",IF(D158="Dólares",C158*Segmentos!$B$4,C158))</f>
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="5" t="n"/>
@@ -3364,6 +4258,11 @@
         <v/>
       </c>
       <c r="H159" s="6" t="n"/>
+      <c r="I159" s="6" t="n"/>
+      <c r="J159" s="7">
+        <f>IF(C159="","",IF(D159="Dólares",C159*Segmentos!$B$4,C159))</f>
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="5" t="n"/>
@@ -3380,6 +4279,11 @@
         <v/>
       </c>
       <c r="H160" s="6" t="n"/>
+      <c r="I160" s="6" t="n"/>
+      <c r="J160" s="7">
+        <f>IF(C160="","",IF(D160="Dólares",C160*Segmentos!$B$4,C160))</f>
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="5" t="n"/>
@@ -3396,6 +4300,11 @@
         <v/>
       </c>
       <c r="H161" s="6" t="n"/>
+      <c r="I161" s="6" t="n"/>
+      <c r="J161" s="7">
+        <f>IF(C161="","",IF(D161="Dólares",C161*Segmentos!$B$4,C161))</f>
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="5" t="n"/>
@@ -3412,6 +4321,11 @@
         <v/>
       </c>
       <c r="H162" s="6" t="n"/>
+      <c r="I162" s="6" t="n"/>
+      <c r="J162" s="7">
+        <f>IF(C162="","",IF(D162="Dólares",C162*Segmentos!$B$4,C162))</f>
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="n"/>
@@ -3428,6 +4342,11 @@
         <v/>
       </c>
       <c r="H163" s="6" t="n"/>
+      <c r="I163" s="6" t="n"/>
+      <c r="J163" s="7">
+        <f>IF(C163="","",IF(D163="Dólares",C163*Segmentos!$B$4,C163))</f>
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="5" t="n"/>
@@ -3444,6 +4363,11 @@
         <v/>
       </c>
       <c r="H164" s="6" t="n"/>
+      <c r="I164" s="6" t="n"/>
+      <c r="J164" s="7">
+        <f>IF(C164="","",IF(D164="Dólares",C164*Segmentos!$B$4,C164))</f>
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="n"/>
@@ -3460,6 +4384,11 @@
         <v/>
       </c>
       <c r="H165" s="6" t="n"/>
+      <c r="I165" s="6" t="n"/>
+      <c r="J165" s="7">
+        <f>IF(C165="","",IF(D165="Dólares",C165*Segmentos!$B$4,C165))</f>
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="5" t="n"/>
@@ -3476,6 +4405,11 @@
         <v/>
       </c>
       <c r="H166" s="6" t="n"/>
+      <c r="I166" s="6" t="n"/>
+      <c r="J166" s="7">
+        <f>IF(C166="","",IF(D166="Dólares",C166*Segmentos!$B$4,C166))</f>
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="n"/>
@@ -3492,6 +4426,11 @@
         <v/>
       </c>
       <c r="H167" s="6" t="n"/>
+      <c r="I167" s="6" t="n"/>
+      <c r="J167" s="7">
+        <f>IF(C167="","",IF(D167="Dólares",C167*Segmentos!$B$4,C167))</f>
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="5" t="n"/>
@@ -3508,6 +4447,11 @@
         <v/>
       </c>
       <c r="H168" s="6" t="n"/>
+      <c r="I168" s="6" t="n"/>
+      <c r="J168" s="7">
+        <f>IF(C168="","",IF(D168="Dólares",C168*Segmentos!$B$4,C168))</f>
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="5" t="n"/>
@@ -3524,6 +4468,11 @@
         <v/>
       </c>
       <c r="H169" s="6" t="n"/>
+      <c r="I169" s="6" t="n"/>
+      <c r="J169" s="7">
+        <f>IF(C169="","",IF(D169="Dólares",C169*Segmentos!$B$4,C169))</f>
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="5" t="n"/>
@@ -3540,6 +4489,11 @@
         <v/>
       </c>
       <c r="H170" s="6" t="n"/>
+      <c r="I170" s="6" t="n"/>
+      <c r="J170" s="7">
+        <f>IF(C170="","",IF(D170="Dólares",C170*Segmentos!$B$4,C170))</f>
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="5" t="n"/>
@@ -3556,6 +4510,11 @@
         <v/>
       </c>
       <c r="H171" s="6" t="n"/>
+      <c r="I171" s="6" t="n"/>
+      <c r="J171" s="7">
+        <f>IF(C171="","",IF(D171="Dólares",C171*Segmentos!$B$4,C171))</f>
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="5" t="n"/>
@@ -3572,6 +4531,11 @@
         <v/>
       </c>
       <c r="H172" s="6" t="n"/>
+      <c r="I172" s="6" t="n"/>
+      <c r="J172" s="7">
+        <f>IF(C172="","",IF(D172="Dólares",C172*Segmentos!$B$4,C172))</f>
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="5" t="n"/>
@@ -3588,6 +4552,11 @@
         <v/>
       </c>
       <c r="H173" s="6" t="n"/>
+      <c r="I173" s="6" t="n"/>
+      <c r="J173" s="7">
+        <f>IF(C173="","",IF(D173="Dólares",C173*Segmentos!$B$4,C173))</f>
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="5" t="n"/>
@@ -3604,6 +4573,11 @@
         <v/>
       </c>
       <c r="H174" s="6" t="n"/>
+      <c r="I174" s="6" t="n"/>
+      <c r="J174" s="7">
+        <f>IF(C174="","",IF(D174="Dólares",C174*Segmentos!$B$4,C174))</f>
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="5" t="n"/>
@@ -3620,6 +4594,11 @@
         <v/>
       </c>
       <c r="H175" s="6" t="n"/>
+      <c r="I175" s="6" t="n"/>
+      <c r="J175" s="7">
+        <f>IF(C175="","",IF(D175="Dólares",C175*Segmentos!$B$4,C175))</f>
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="5" t="n"/>
@@ -3636,6 +4615,11 @@
         <v/>
       </c>
       <c r="H176" s="6" t="n"/>
+      <c r="I176" s="6" t="n"/>
+      <c r="J176" s="7">
+        <f>IF(C176="","",IF(D176="Dólares",C176*Segmentos!$B$4,C176))</f>
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="5" t="n"/>
@@ -3652,6 +4636,11 @@
         <v/>
       </c>
       <c r="H177" s="6" t="n"/>
+      <c r="I177" s="6" t="n"/>
+      <c r="J177" s="7">
+        <f>IF(C177="","",IF(D177="Dólares",C177*Segmentos!$B$4,C177))</f>
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n"/>
@@ -3668,6 +4657,11 @@
         <v/>
       </c>
       <c r="H178" s="6" t="n"/>
+      <c r="I178" s="6" t="n"/>
+      <c r="J178" s="7">
+        <f>IF(C178="","",IF(D178="Dólares",C178*Segmentos!$B$4,C178))</f>
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="5" t="n"/>
@@ -3684,6 +4678,11 @@
         <v/>
       </c>
       <c r="H179" s="6" t="n"/>
+      <c r="I179" s="6" t="n"/>
+      <c r="J179" s="7">
+        <f>IF(C179="","",IF(D179="Dólares",C179*Segmentos!$B$4,C179))</f>
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="5" t="n"/>
@@ -3700,6 +4699,11 @@
         <v/>
       </c>
       <c r="H180" s="6" t="n"/>
+      <c r="I180" s="6" t="n"/>
+      <c r="J180" s="7">
+        <f>IF(C180="","",IF(D180="Dólares",C180*Segmentos!$B$4,C180))</f>
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="5" t="n"/>
@@ -3716,6 +4720,11 @@
         <v/>
       </c>
       <c r="H181" s="6" t="n"/>
+      <c r="I181" s="6" t="n"/>
+      <c r="J181" s="7">
+        <f>IF(C181="","",IF(D181="Dólares",C181*Segmentos!$B$4,C181))</f>
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n"/>
@@ -3732,6 +4741,11 @@
         <v/>
       </c>
       <c r="H182" s="6" t="n"/>
+      <c r="I182" s="6" t="n"/>
+      <c r="J182" s="7">
+        <f>IF(C182="","",IF(D182="Dólares",C182*Segmentos!$B$4,C182))</f>
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n"/>
@@ -3748,6 +4762,11 @@
         <v/>
       </c>
       <c r="H183" s="6" t="n"/>
+      <c r="I183" s="6" t="n"/>
+      <c r="J183" s="7">
+        <f>IF(C183="","",IF(D183="Dólares",C183*Segmentos!$B$4,C183))</f>
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="5" t="n"/>
@@ -3764,6 +4783,11 @@
         <v/>
       </c>
       <c r="H184" s="6" t="n"/>
+      <c r="I184" s="6" t="n"/>
+      <c r="J184" s="7">
+        <f>IF(C184="","",IF(D184="Dólares",C184*Segmentos!$B$4,C184))</f>
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="5" t="n"/>
@@ -3780,6 +4804,11 @@
         <v/>
       </c>
       <c r="H185" s="6" t="n"/>
+      <c r="I185" s="6" t="n"/>
+      <c r="J185" s="7">
+        <f>IF(C185="","",IF(D185="Dólares",C185*Segmentos!$B$4,C185))</f>
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n"/>
@@ -3796,6 +4825,11 @@
         <v/>
       </c>
       <c r="H186" s="6" t="n"/>
+      <c r="I186" s="6" t="n"/>
+      <c r="J186" s="7">
+        <f>IF(C186="","",IF(D186="Dólares",C186*Segmentos!$B$4,C186))</f>
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n"/>
@@ -3812,6 +4846,11 @@
         <v/>
       </c>
       <c r="H187" s="6" t="n"/>
+      <c r="I187" s="6" t="n"/>
+      <c r="J187" s="7">
+        <f>IF(C187="","",IF(D187="Dólares",C187*Segmentos!$B$4,C187))</f>
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n"/>
@@ -3828,6 +4867,11 @@
         <v/>
       </c>
       <c r="H188" s="6" t="n"/>
+      <c r="I188" s="6" t="n"/>
+      <c r="J188" s="7">
+        <f>IF(C188="","",IF(D188="Dólares",C188*Segmentos!$B$4,C188))</f>
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n"/>
@@ -3844,6 +4888,11 @@
         <v/>
       </c>
       <c r="H189" s="6" t="n"/>
+      <c r="I189" s="6" t="n"/>
+      <c r="J189" s="7">
+        <f>IF(C189="","",IF(D189="Dólares",C189*Segmentos!$B$4,C189))</f>
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n"/>
@@ -3860,6 +4909,11 @@
         <v/>
       </c>
       <c r="H190" s="6" t="n"/>
+      <c r="I190" s="6" t="n"/>
+      <c r="J190" s="7">
+        <f>IF(C190="","",IF(D190="Dólares",C190*Segmentos!$B$4,C190))</f>
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="5" t="n"/>
@@ -3876,6 +4930,11 @@
         <v/>
       </c>
       <c r="H191" s="6" t="n"/>
+      <c r="I191" s="6" t="n"/>
+      <c r="J191" s="7">
+        <f>IF(C191="","",IF(D191="Dólares",C191*Segmentos!$B$4,C191))</f>
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="5" t="n"/>
@@ -3892,6 +4951,11 @@
         <v/>
       </c>
       <c r="H192" s="6" t="n"/>
+      <c r="I192" s="6" t="n"/>
+      <c r="J192" s="7">
+        <f>IF(C192="","",IF(D192="Dólares",C192*Segmentos!$B$4,C192))</f>
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n"/>
@@ -3908,6 +4972,11 @@
         <v/>
       </c>
       <c r="H193" s="6" t="n"/>
+      <c r="I193" s="6" t="n"/>
+      <c r="J193" s="7">
+        <f>IF(C193="","",IF(D193="Dólares",C193*Segmentos!$B$4,C193))</f>
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n"/>
@@ -3924,6 +4993,11 @@
         <v/>
       </c>
       <c r="H194" s="6" t="n"/>
+      <c r="I194" s="6" t="n"/>
+      <c r="J194" s="7">
+        <f>IF(C194="","",IF(D194="Dólares",C194*Segmentos!$B$4,C194))</f>
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="5" t="n"/>
@@ -3940,6 +5014,11 @@
         <v/>
       </c>
       <c r="H195" s="6" t="n"/>
+      <c r="I195" s="6" t="n"/>
+      <c r="J195" s="7">
+        <f>IF(C195="","",IF(D195="Dólares",C195*Segmentos!$B$4,C195))</f>
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="5" t="n"/>
@@ -3956,6 +5035,11 @@
         <v/>
       </c>
       <c r="H196" s="6" t="n"/>
+      <c r="I196" s="6" t="n"/>
+      <c r="J196" s="7">
+        <f>IF(C196="","",IF(D196="Dólares",C196*Segmentos!$B$4,C196))</f>
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n"/>
@@ -3972,6 +5056,11 @@
         <v/>
       </c>
       <c r="H197" s="6" t="n"/>
+      <c r="I197" s="6" t="n"/>
+      <c r="J197" s="7">
+        <f>IF(C197="","",IF(D197="Dólares",C197*Segmentos!$B$4,C197))</f>
+        <v/>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="5" t="n"/>
@@ -3988,6 +5077,11 @@
         <v/>
       </c>
       <c r="H198" s="6" t="n"/>
+      <c r="I198" s="6" t="n"/>
+      <c r="J198" s="7">
+        <f>IF(C198="","",IF(D198="Dólares",C198*Segmentos!$B$4,C198))</f>
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n"/>
@@ -4004,6 +5098,11 @@
         <v/>
       </c>
       <c r="H199" s="6" t="n"/>
+      <c r="I199" s="6" t="n"/>
+      <c r="J199" s="7">
+        <f>IF(C199="","",IF(D199="Dólares",C199*Segmentos!$B$4,C199))</f>
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n"/>
@@ -4020,9 +5119,14 @@
         <v/>
       </c>
       <c r="H200" s="6" t="n"/>
+      <c r="I200" s="6" t="n"/>
+      <c r="J200" s="7">
+        <f>IF(C200="","",IF(D200="Dólares",C200*Segmentos!$B$4,C200))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"iO,BBVA,pareja"</formula1>
     </dataValidation>
@@ -4031,6 +5135,9 @@
     </dataValidation>
     <dataValidation sqref="H2:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,Pagado"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Comida,Transporte,Ropa y compras,Ocio,Suscripciones,Pareja,Otros"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4138,7 +5245,757 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Gasto por segmento y ciclo de tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Ingreso mensual (S/)</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>← escribe tu ingreso mensual</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Tipo de cambio (S/ por US$)</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>← referencial, ajústalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Fecha de Pago</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Ropa y compras</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Ocio</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Suscripciones</t>
+        </is>
+      </c>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>Total S/</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>% del ingreso</t>
+        </is>
+      </c>
+      <c r="M6" s="18" t="inlineStr">
+        <is>
+          <t>Aprox. al cierre S/</t>
+        </is>
+      </c>
+      <c r="N6" s="18" t="inlineStr">
+        <is>
+          <t>% aprox. del ingreso</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19">
+        <f>DATE(2026,11,5)</f>
+        <v/>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C7" s="21">
+        <f>IF(OR(A7="",B7="pareja"),"",DATE(YEAR(A7),MONTH(A7)-1,IF(B7="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D7" s="22">
+        <f>IF($A7="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A7,Gastos!$E:$E,$B7,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E7" s="22">
+        <f>IF($A7="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A7,Gastos!$E:$E,$B7,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F7" s="22">
+        <f>IF($A7="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A7,Gastos!$E:$E,$B7,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G7" s="22">
+        <f>IF($A7="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A7,Gastos!$E:$E,$B7,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H7" s="22">
+        <f>IF($A7="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A7,Gastos!$E:$E,$B7,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I7" s="22">
+        <f>IF($A7="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A7,Gastos!$E:$E,$B7,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J7" s="22">
+        <f>IF($A7="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A7,Gastos!$E:$E,$B7,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K7" s="22">
+        <f>IF(A7="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A7,Gastos!$E:$E,$B7))</f>
+        <v/>
+      </c>
+      <c r="L7" s="23">
+        <f>IF(OR(A7="",$B$3=""),"",K7/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M7" s="22">
+        <f>IF(A7="","",IF(OR(C7="",TODAY()&gt;=C7),K7,K7/MAX(1,TODAY()-(EDATE(C7,-1)+1)+1)*(C7-(EDATE(C7,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N7" s="23">
+        <f>IF(OR(A7="",$B$3=""),"",M7/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19">
+        <f>DATE(2026,11,12)</f>
+        <v/>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>iO</t>
+        </is>
+      </c>
+      <c r="C8" s="21">
+        <f>IF(OR(A8="",B8="pareja"),"",DATE(YEAR(A8),MONTH(A8)-1,IF(B8="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D8" s="22">
+        <f>IF($A8="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A8,Gastos!$E:$E,$B8,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E8" s="22">
+        <f>IF($A8="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A8,Gastos!$E:$E,$B8,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F8" s="22">
+        <f>IF($A8="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A8,Gastos!$E:$E,$B8,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G8" s="22">
+        <f>IF($A8="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A8,Gastos!$E:$E,$B8,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H8" s="22">
+        <f>IF($A8="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A8,Gastos!$E:$E,$B8,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I8" s="22">
+        <f>IF($A8="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A8,Gastos!$E:$E,$B8,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J8" s="22">
+        <f>IF($A8="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A8,Gastos!$E:$E,$B8,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K8" s="22">
+        <f>IF(A8="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A8,Gastos!$E:$E,$B8))</f>
+        <v/>
+      </c>
+      <c r="L8" s="23">
+        <f>IF(OR(A8="",$B$3=""),"",K8/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M8" s="22">
+        <f>IF(A8="","",IF(OR(C8="",TODAY()&gt;=C8),K8,K8/MAX(1,TODAY()-(EDATE(C8,-1)+1)+1)*(C8-(EDATE(C8,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N8" s="23">
+        <f>IF(OR(A8="",$B$3=""),"",M8/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19">
+        <f>DATE(2026,11,20)</f>
+        <v/>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>pareja</t>
+        </is>
+      </c>
+      <c r="C9" s="21">
+        <f>IF(OR(A9="",B9="pareja"),"",DATE(YEAR(A9),MONTH(A9)-1,IF(B9="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D9" s="22">
+        <f>IF($A9="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A9,Gastos!$E:$E,$B9,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E9" s="22">
+        <f>IF($A9="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A9,Gastos!$E:$E,$B9,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F9" s="22">
+        <f>IF($A9="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A9,Gastos!$E:$E,$B9,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G9" s="22">
+        <f>IF($A9="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A9,Gastos!$E:$E,$B9,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H9" s="22">
+        <f>IF($A9="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A9,Gastos!$E:$E,$B9,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I9" s="22">
+        <f>IF($A9="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A9,Gastos!$E:$E,$B9,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J9" s="22">
+        <f>IF($A9="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A9,Gastos!$E:$E,$B9,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K9" s="22">
+        <f>IF(A9="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A9,Gastos!$E:$E,$B9))</f>
+        <v/>
+      </c>
+      <c r="L9" s="23">
+        <f>IF(OR(A9="",$B$3=""),"",K9/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M9" s="22">
+        <f>IF(A9="","",IF(OR(C9="",TODAY()&gt;=C9),K9,K9/MAX(1,TODAY()-(EDATE(C9,-1)+1)+1)*(C9-(EDATE(C9,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N9" s="23">
+        <f>IF(OR(A9="",$B$3=""),"",M9/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="20" t="n"/>
+      <c r="C10" s="21">
+        <f>IF(OR(A10="",B10="pareja"),"",DATE(YEAR(A10),MONTH(A10)-1,IF(B10="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D10" s="22">
+        <f>IF($A10="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A10,Gastos!$E:$E,$B10,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E10" s="22">
+        <f>IF($A10="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A10,Gastos!$E:$E,$B10,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F10" s="22">
+        <f>IF($A10="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A10,Gastos!$E:$E,$B10,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G10" s="22">
+        <f>IF($A10="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A10,Gastos!$E:$E,$B10,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>IF($A10="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A10,Gastos!$E:$E,$B10,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I10" s="22">
+        <f>IF($A10="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A10,Gastos!$E:$E,$B10,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J10" s="22">
+        <f>IF($A10="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A10,Gastos!$E:$E,$B10,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K10" s="22">
+        <f>IF(A10="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A10,Gastos!$E:$E,$B10))</f>
+        <v/>
+      </c>
+      <c r="L10" s="23">
+        <f>IF(OR(A10="",$B$3=""),"",K10/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M10" s="22">
+        <f>IF(A10="","",IF(OR(C10="",TODAY()&gt;=C10),K10,K10/MAX(1,TODAY()-(EDATE(C10,-1)+1)+1)*(C10-(EDATE(C10,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N10" s="23">
+        <f>IF(OR(A10="",$B$3=""),"",M10/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="20" t="n"/>
+      <c r="C11" s="21">
+        <f>IF(OR(A11="",B11="pareja"),"",DATE(YEAR(A11),MONTH(A11)-1,IF(B11="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D11" s="22">
+        <f>IF($A11="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A11,Gastos!$E:$E,$B11,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E11" s="22">
+        <f>IF($A11="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A11,Gastos!$E:$E,$B11,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F11" s="22">
+        <f>IF($A11="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A11,Gastos!$E:$E,$B11,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G11" s="22">
+        <f>IF($A11="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A11,Gastos!$E:$E,$B11,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H11" s="22">
+        <f>IF($A11="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A11,Gastos!$E:$E,$B11,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I11" s="22">
+        <f>IF($A11="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A11,Gastos!$E:$E,$B11,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J11" s="22">
+        <f>IF($A11="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A11,Gastos!$E:$E,$B11,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K11" s="22">
+        <f>IF(A11="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A11,Gastos!$E:$E,$B11))</f>
+        <v/>
+      </c>
+      <c r="L11" s="23">
+        <f>IF(OR(A11="",$B$3=""),"",K11/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M11" s="22">
+        <f>IF(A11="","",IF(OR(C11="",TODAY()&gt;=C11),K11,K11/MAX(1,TODAY()-(EDATE(C11,-1)+1)+1)*(C11-(EDATE(C11,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N11" s="23">
+        <f>IF(OR(A11="",$B$3=""),"",M11/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="20" t="n"/>
+      <c r="C12" s="21">
+        <f>IF(OR(A12="",B12="pareja"),"",DATE(YEAR(A12),MONTH(A12)-1,IF(B12="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D12" s="22">
+        <f>IF($A12="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A12,Gastos!$E:$E,$B12,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E12" s="22">
+        <f>IF($A12="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A12,Gastos!$E:$E,$B12,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F12" s="22">
+        <f>IF($A12="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A12,Gastos!$E:$E,$B12,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G12" s="22">
+        <f>IF($A12="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A12,Gastos!$E:$E,$B12,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H12" s="22">
+        <f>IF($A12="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A12,Gastos!$E:$E,$B12,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I12" s="22">
+        <f>IF($A12="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A12,Gastos!$E:$E,$B12,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J12" s="22">
+        <f>IF($A12="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A12,Gastos!$E:$E,$B12,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K12" s="22">
+        <f>IF(A12="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A12,Gastos!$E:$E,$B12))</f>
+        <v/>
+      </c>
+      <c r="L12" s="23">
+        <f>IF(OR(A12="",$B$3=""),"",K12/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M12" s="22">
+        <f>IF(A12="","",IF(OR(C12="",TODAY()&gt;=C12),K12,K12/MAX(1,TODAY()-(EDATE(C12,-1)+1)+1)*(C12-(EDATE(C12,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N12" s="23">
+        <f>IF(OR(A12="",$B$3=""),"",M12/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="20" t="n"/>
+      <c r="C13" s="21">
+        <f>IF(OR(A13="",B13="pareja"),"",DATE(YEAR(A13),MONTH(A13)-1,IF(B13="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D13" s="22">
+        <f>IF($A13="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A13,Gastos!$E:$E,$B13,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E13" s="22">
+        <f>IF($A13="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A13,Gastos!$E:$E,$B13,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F13" s="22">
+        <f>IF($A13="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A13,Gastos!$E:$E,$B13,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G13" s="22">
+        <f>IF($A13="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A13,Gastos!$E:$E,$B13,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H13" s="22">
+        <f>IF($A13="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A13,Gastos!$E:$E,$B13,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I13" s="22">
+        <f>IF($A13="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A13,Gastos!$E:$E,$B13,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J13" s="22">
+        <f>IF($A13="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A13,Gastos!$E:$E,$B13,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K13" s="22">
+        <f>IF(A13="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A13,Gastos!$E:$E,$B13))</f>
+        <v/>
+      </c>
+      <c r="L13" s="23">
+        <f>IF(OR(A13="",$B$3=""),"",K13/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M13" s="22">
+        <f>IF(A13="","",IF(OR(C13="",TODAY()&gt;=C13),K13,K13/MAX(1,TODAY()-(EDATE(C13,-1)+1)+1)*(C13-(EDATE(C13,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N13" s="23">
+        <f>IF(OR(A13="",$B$3=""),"",M13/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="20" t="n"/>
+      <c r="C14" s="21">
+        <f>IF(OR(A14="",B14="pareja"),"",DATE(YEAR(A14),MONTH(A14)-1,IF(B14="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D14" s="22">
+        <f>IF($A14="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A14,Gastos!$E:$E,$B14,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E14" s="22">
+        <f>IF($A14="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A14,Gastos!$E:$E,$B14,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F14" s="22">
+        <f>IF($A14="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A14,Gastos!$E:$E,$B14,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G14" s="22">
+        <f>IF($A14="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A14,Gastos!$E:$E,$B14,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H14" s="22">
+        <f>IF($A14="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A14,Gastos!$E:$E,$B14,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I14" s="22">
+        <f>IF($A14="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A14,Gastos!$E:$E,$B14,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J14" s="22">
+        <f>IF($A14="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A14,Gastos!$E:$E,$B14,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K14" s="22">
+        <f>IF(A14="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A14,Gastos!$E:$E,$B14))</f>
+        <v/>
+      </c>
+      <c r="L14" s="23">
+        <f>IF(OR(A14="",$B$3=""),"",K14/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M14" s="22">
+        <f>IF(A14="","",IF(OR(C14="",TODAY()&gt;=C14),K14,K14/MAX(1,TODAY()-(EDATE(C14,-1)+1)+1)*(C14-(EDATE(C14,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N14" s="23">
+        <f>IF(OR(A14="",$B$3=""),"",M14/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="20" t="n"/>
+      <c r="C15" s="21">
+        <f>IF(OR(A15="",B15="pareja"),"",DATE(YEAR(A15),MONTH(A15)-1,IF(B15="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D15" s="22">
+        <f>IF($A15="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A15,Gastos!$E:$E,$B15,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E15" s="22">
+        <f>IF($A15="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A15,Gastos!$E:$E,$B15,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F15" s="22">
+        <f>IF($A15="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A15,Gastos!$E:$E,$B15,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G15" s="22">
+        <f>IF($A15="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A15,Gastos!$E:$E,$B15,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H15" s="22">
+        <f>IF($A15="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A15,Gastos!$E:$E,$B15,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I15" s="22">
+        <f>IF($A15="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A15,Gastos!$E:$E,$B15,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J15" s="22">
+        <f>IF($A15="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A15,Gastos!$E:$E,$B15,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K15" s="22">
+        <f>IF(A15="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A15,Gastos!$E:$E,$B15))</f>
+        <v/>
+      </c>
+      <c r="L15" s="23">
+        <f>IF(OR(A15="",$B$3=""),"",K15/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M15" s="22">
+        <f>IF(A15="","",IF(OR(C15="",TODAY()&gt;=C15),K15,K15/MAX(1,TODAY()-(EDATE(C15,-1)+1)+1)*(C15-(EDATE(C15,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N15" s="23">
+        <f>IF(OR(A15="",$B$3=""),"",M15/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="20" t="n"/>
+      <c r="C16" s="21">
+        <f>IF(OR(A16="",B16="pareja"),"",DATE(YEAR(A16),MONTH(A16)-1,IF(B16="iO",25,10)))</f>
+        <v/>
+      </c>
+      <c r="D16" s="22">
+        <f>IF($A16="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A16,Gastos!$E:$E,$B16,Gastos!$I:$I,D$6))</f>
+        <v/>
+      </c>
+      <c r="E16" s="22">
+        <f>IF($A16="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A16,Gastos!$E:$E,$B16,Gastos!$I:$I,E$6))</f>
+        <v/>
+      </c>
+      <c r="F16" s="22">
+        <f>IF($A16="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A16,Gastos!$E:$E,$B16,Gastos!$I:$I,F$6))</f>
+        <v/>
+      </c>
+      <c r="G16" s="22">
+        <f>IF($A16="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A16,Gastos!$E:$E,$B16,Gastos!$I:$I,G$6))</f>
+        <v/>
+      </c>
+      <c r="H16" s="22">
+        <f>IF($A16="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A16,Gastos!$E:$E,$B16,Gastos!$I:$I,H$6))</f>
+        <v/>
+      </c>
+      <c r="I16" s="22">
+        <f>IF($A16="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A16,Gastos!$E:$E,$B16,Gastos!$I:$I,I$6))</f>
+        <v/>
+      </c>
+      <c r="J16" s="22">
+        <f>IF($A16="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A16,Gastos!$E:$E,$B16,Gastos!$I:$I,J$6))</f>
+        <v/>
+      </c>
+      <c r="K16" s="22">
+        <f>IF(A16="","",SUMIFS(Gastos!$J:$J,Gastos!$G:$G,$A16,Gastos!$E:$E,$B16))</f>
+        <v/>
+      </c>
+      <c r="L16" s="23">
+        <f>IF(OR(A16="",$B$3=""),"",K16/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M16" s="22">
+        <f>IF(A16="","",IF(OR(C16="",TODAY()&gt;=C16),K16,K16/MAX(1,TODAY()-(EDATE(C16,-1)+1)+1)*(C16-(EDATE(C16,-1)+1)+1)))</f>
+        <v/>
+      </c>
+      <c r="N16" s="23">
+        <f>IF(OR(A16="",$B$3=""),"",M16/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="n"/>
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="25">
+        <f>SUM(D7:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="25">
+        <f>SUM(E7:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="25">
+        <f>SUM(F7:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="25">
+        <f>SUM(G7:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="25">
+        <f>SUM(H7:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="25">
+        <f>SUM(I7:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="25">
+        <f>SUM(J7:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="25">
+        <f>SUM(K7:K16)</f>
+        <v/>
+      </c>
+      <c r="L17" s="26">
+        <f>IF($B$3="","",K17/$B$3)</f>
+        <v/>
+      </c>
+      <c r="M17" s="25">
+        <f>SUM(M7:M16)</f>
+        <v/>
+      </c>
+      <c r="N17" s="26">
+        <f>IF($B$3="","",M17/$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Los montos en dólares se convierten con el tipo de cambio de B4. 'Aprox. al cierre' proyecta el ritmo diario del ciclo hasta el corte (más confiable a mitad de ciclo que al inicio).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>Para agregar otro ciclo, escribe su Fecha de Pago y Tarjeta en las celdas amarillas libres de arriba.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B7:B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"iO,BBVA,pareja"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -4282,6 +6139,20 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>5) Segmentos: en 'Gastos' elige el Segmento de cada gasto (lista desplegable). La pestaña 'Segmentos' resume por ciclo de tarjeta:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   total por segmento, % de tu ingreso y un aproximado de lo que gastarás al corte. Llena tu ingreso (B3) y el tipo de cambio (B4).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar consumos BBVA del 11 de octubre
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Un1EUwZaDgQpX57Ncqbdo
</commit_message>
<xml_diff>
--- a/Seguimiento_Gastos.xlsx
+++ b/Seguimiento_Gastos.xlsx
@@ -1262,11 +1262,27 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
+      <c r="A17" s="5" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>GlobalE /Ralph La</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
       <c r="F17" s="5">
         <f>IF(A17="","",IF(DAY(A17)&lt;=IF(E17="iO",25,10),DATE(YEAR(A17),MONTH(A17),IF(E17="iO",25,10)),DATE(YEAR(A17),MONTH(A17)+1,IF(E17="iO",25,10))))</f>
         <v/>
@@ -1275,19 +1291,43 @@
         <f>IF(F17="","",DATE(YEAR(F17),MONTH(F17)+1,IF(E17="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>Ropa y compras</t>
+        </is>
+      </c>
       <c r="J17" s="7">
         <f>IF(C17="","",IF(D17="Dólares",C17*Segmentos!$B$4,C17))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
+      <c r="A18" s="5" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>ANTHROPIC* CLAUDE</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Dólares</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
       <c r="F18" s="5">
         <f>IF(A18="","",IF(DAY(A18)&lt;=IF(E18="iO",25,10),DATE(YEAR(A18),MONTH(A18),IF(E18="iO",25,10)),DATE(YEAR(A18),MONTH(A18)+1,IF(E18="iO",25,10))))</f>
         <v/>
@@ -1296,19 +1336,43 @@
         <f>IF(F18="","",DATE(YEAR(F18),MONTH(F18)+1,IF(E18="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="n"/>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>Suscripciones</t>
+        </is>
+      </c>
       <c r="J18" s="7">
         <f>IF(C18="","",IF(D18="Dólares",C18*Segmentos!$B$4,C18))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
+      <c r="A19" s="5" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>LA LENA MALL DE C</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
       <c r="F19" s="5">
         <f>IF(A19="","",IF(DAY(A19)&lt;=IF(E19="iO",25,10),DATE(YEAR(A19),MONTH(A19),IF(E19="iO",25,10)),DATE(YEAR(A19),MONTH(A19)+1,IF(E19="iO",25,10))))</f>
         <v/>
@@ -1317,19 +1381,43 @@
         <f>IF(F19="","",DATE(YEAR(F19),MONTH(F19)+1,IF(E19="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H19" s="6" t="n"/>
-      <c r="I19" s="6" t="n"/>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
       <c r="J19" s="7">
         <f>IF(C19="","",IF(D19="Dólares",C19*Segmentos!$B$4,C19))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
+      <c r="A20" s="5" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>LIDERMAN PARKING</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Soles</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
       <c r="F20" s="5">
         <f>IF(A20="","",IF(DAY(A20)&lt;=IF(E20="iO",25,10),DATE(YEAR(A20),MONTH(A20),IF(E20="iO",25,10)),DATE(YEAR(A20),MONTH(A20)+1,IF(E20="iO",25,10))))</f>
         <v/>
@@ -1338,8 +1426,16 @@
         <f>IF(F20="","",DATE(YEAR(F20),MONTH(F20)+1,IF(E20="iO",12,5)))</f>
         <v/>
       </c>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
       <c r="J20" s="7">
         <f>IF(C20="","",IF(D20="Dólares",C20*Segmentos!$B$4,C20))</f>
         <v/>
@@ -5549,8 +5645,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="20" t="n"/>
+      <c r="A10" s="19">
+        <f>DATE(2026,12,5)</f>
+        <v/>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
       <c r="C10" s="21">
         <f>IF(OR(A10="",B10="pareja"),"",DATE(YEAR(A10),MONTH(A10)-1,IF(B10="iO",25,10)))</f>
         <v/>

</xml_diff>